<commit_message>
Current working state before testing QB vs defense feature
</commit_message>
<xml_diff>
--- a/data/bets-and-clv.xlsx
+++ b/data/bets-and-clv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/98038a0616e2a1bf/Desktop/Development/Projects/nfl-prop-model-2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="373" documentId="8_{1CC852AD-96B9-495C-9858-3FDD56D405B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{654574DC-FF9A-447B-BE5E-2D4699580F1F}"/>
+  <xr:revisionPtr revIDLastSave="420" documentId="8_{1CC852AD-96B9-495C-9858-3FDD56D405B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD24EC2B-9CE2-48F3-838C-0ECC9A27C52A}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{3786BA1E-DAAC-4214-853F-3F41588D39A2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="71">
   <si>
     <t>Date</t>
   </si>
@@ -231,6 +231,24 @@
   </si>
   <si>
     <t>PHI vs. NYG</t>
+  </si>
+  <si>
+    <t>J.Herbert</t>
+  </si>
+  <si>
+    <t>LAC vs.MIA</t>
+  </si>
+  <si>
+    <t>DEN vs. NYJ</t>
+  </si>
+  <si>
+    <t>J.Fields</t>
+  </si>
+  <si>
+    <t>DAL vs. CAR</t>
+  </si>
+  <si>
+    <t>IND vs. ARI</t>
   </si>
 </sst>
 </file>
@@ -294,7 +312,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -323,9 +341,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -711,7 +726,7 @@
     <col min="2" max="2" width="13.6796875" customWidth="1"/>
     <col min="3" max="3" width="11.1328125" customWidth="1"/>
     <col min="4" max="4" width="11.1796875" customWidth="1"/>
-    <col min="10" max="10" width="8.7265625" style="23"/>
+    <col min="10" max="10" width="8.7265625" style="22"/>
     <col min="11" max="11" width="8.7265625" style="10"/>
     <col min="12" max="12" width="9.31640625" customWidth="1"/>
     <col min="14" max="14" width="8.7265625" style="10"/>
@@ -719,7 +734,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="29.5" x14ac:dyDescent="0.75">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -746,7 +761,7 @@
       <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="22" t="s">
+      <c r="J1" s="21" t="s">
         <v>7</v>
       </c>
       <c r="K1" s="9" t="s">
@@ -796,7 +811,7 @@
       <c r="I2">
         <v>-112</v>
       </c>
-      <c r="J2" s="23">
+      <c r="J2" s="22">
         <f>IF(E2="Over", H2-F2, IF(E2="Under", F2-H2, ""))</f>
         <v>-6</v>
       </c>
@@ -845,7 +860,7 @@
       <c r="I3">
         <v>-111</v>
       </c>
-      <c r="J3" s="23">
+      <c r="J3" s="22">
         <f t="shared" ref="J3:J20" si="0">IF(E3="Over", H3-F3, IF(E3="Under", F3-H3, ""))</f>
         <v>10</v>
       </c>
@@ -890,7 +905,7 @@
       <c r="I4">
         <v>-112</v>
       </c>
-      <c r="J4" s="23">
+      <c r="J4" s="22">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
@@ -935,7 +950,7 @@
       <c r="I5">
         <v>-112</v>
       </c>
-      <c r="J5" s="23">
+      <c r="J5" s="22">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -980,7 +995,7 @@
       <c r="I6">
         <v>-112</v>
       </c>
-      <c r="J6" s="23">
+      <c r="J6" s="22">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -1025,7 +1040,7 @@
       <c r="I7">
         <v>-111</v>
       </c>
-      <c r="J7" s="23">
+      <c r="J7" s="22">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -1070,7 +1085,7 @@
       <c r="I8">
         <v>-110</v>
       </c>
-      <c r="J8" s="23">
+      <c r="J8" s="22">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -1115,7 +1130,7 @@
       <c r="I9">
         <v>-112</v>
       </c>
-      <c r="J9" s="23">
+      <c r="J9" s="22">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -1160,7 +1175,7 @@
       <c r="I10">
         <v>-112</v>
       </c>
-      <c r="J10" s="23">
+      <c r="J10" s="22">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1205,7 +1220,7 @@
       <c r="I11">
         <v>-112</v>
       </c>
-      <c r="J11" s="23">
+      <c r="J11" s="22">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -1250,7 +1265,7 @@
       <c r="I12">
         <v>-112</v>
       </c>
-      <c r="J12" s="23">
+      <c r="J12" s="22">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -1295,7 +1310,7 @@
       <c r="I13">
         <v>-111</v>
       </c>
-      <c r="J13" s="23">
+      <c r="J13" s="22">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
@@ -1340,7 +1355,7 @@
       <c r="I14">
         <v>-113</v>
       </c>
-      <c r="J14" s="23">
+      <c r="J14" s="22">
         <f t="shared" si="0"/>
         <v>-1</v>
       </c>
@@ -1386,7 +1401,7 @@
       <c r="I15">
         <v>-113</v>
       </c>
-      <c r="J15" s="23">
+      <c r="J15" s="22">
         <f t="shared" si="0"/>
         <v>-3</v>
       </c>
@@ -1432,7 +1447,7 @@
       <c r="I16" s="2">
         <v>-111</v>
       </c>
-      <c r="J16" s="23">
+      <c r="J16" s="22">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
@@ -1477,7 +1492,7 @@
       <c r="I17" s="2">
         <v>-110</v>
       </c>
-      <c r="J17" s="23">
+      <c r="J17" s="22">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
@@ -1522,7 +1537,7 @@
       <c r="I18">
         <v>-113</v>
       </c>
-      <c r="J18" s="23">
+      <c r="J18" s="22">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -1567,7 +1582,7 @@
       <c r="I19">
         <v>-125</v>
       </c>
-      <c r="J19" s="23">
+      <c r="J19" s="22">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
@@ -1612,7 +1627,7 @@
       <c r="I20">
         <v>-110</v>
       </c>
-      <c r="J20" s="23">
+      <c r="J20" s="22">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -1653,207 +1668,279 @@
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="C22" s="5"/>
+      <c r="A22" s="3">
+        <v>45937</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" t="s">
+        <v>66</v>
+      </c>
+      <c r="E22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22">
+        <v>250.5</v>
+      </c>
+      <c r="G22">
+        <v>-111</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A23" s="12"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-    </row>
-    <row r="25" spans="1:14" ht="24.25" x14ac:dyDescent="0.75">
-      <c r="A25" s="14"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A26" s="15"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A27" s="1" t="s">
+      <c r="A23" s="3">
+        <v>45937</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D23" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23">
+        <v>196.5</v>
+      </c>
+      <c r="G23">
+        <v>-113</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.75">
+      <c r="A24" s="3">
+        <v>45938</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" t="s">
+        <v>70</v>
+      </c>
+      <c r="E24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24">
+        <v>234.5</v>
+      </c>
+      <c r="G24">
+        <v>-113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.75">
+      <c r="A25" s="3">
+        <v>45939</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" t="s">
+        <v>69</v>
+      </c>
+      <c r="E25" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25">
+        <v>245.5</v>
+      </c>
+      <c r="G25">
+        <v>-113</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.75">
+      <c r="A29" s="14"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.75">
+      <c r="A30" s="16"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.75">
+      <c r="A31" s="16"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.75">
+      <c r="A32" s="16"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A33" s="17"/>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A34" s="17"/>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A35" s="17"/>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A36" s="16"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A37" s="14"/>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A38" s="15"/>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A39" s="14"/>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A40" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B40" s="25" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A28" s="23">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A41" s="22">
         <f>AVERAGE(J2:J100)</f>
         <v>3.5789473684210527</v>
       </c>
-      <c r="B28" s="25">
+      <c r="B41" s="24">
         <f>COUNTIF(J2:J100,"&gt;0") / COUNTA(J2:J100)</f>
         <v>0.78947368421052633</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A29" s="15"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A30" s="17"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A31" s="17"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A32" s="17"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A33" s="18"/>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A34" s="18"/>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A35" s="18"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A36" s="17"/>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A37" s="15"/>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A38" s="16"/>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A39" s="15"/>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A40" s="15"/>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A41" s="17"/>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A42" s="18"/>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A43" s="18"/>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A44" s="19"/>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A45" s="19"/>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A46" s="19"/>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A47" s="15"/>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A48" s="16"/>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A42" s="17"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A43" s="17"/>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A44" s="18"/>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A45" s="18"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A46" s="18"/>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A47" s="14"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A48" s="15"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A49" s="15"/>
+      <c r="A49" s="14"/>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A50" s="15"/>
+      <c r="A50" s="14"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A51" s="17"/>
+      <c r="A51" s="16"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A52" s="18"/>
+      <c r="A52" s="17"/>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A53" s="18"/>
+      <c r="A53" s="17"/>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A54" s="17"/>
+      <c r="A54" s="16"/>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A55" s="15"/>
+      <c r="A55" s="14"/>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A56" s="16"/>
+      <c r="A56" s="15"/>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A57" s="15"/>
+      <c r="A57" s="14"/>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A58" s="15"/>
+      <c r="A58" s="14"/>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A59" s="20"/>
+      <c r="A59" s="19"/>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A60" s="20"/>
+      <c r="A60" s="19"/>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A61" s="20"/>
+      <c r="A61" s="19"/>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A62" s="20"/>
+      <c r="A62" s="19"/>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A63" s="20"/>
+      <c r="A63" s="19"/>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A64" s="17"/>
+      <c r="A64" s="16"/>
     </row>
     <row r="66" spans="1:1" ht="24.25" x14ac:dyDescent="0.75">
-      <c r="A66" s="14"/>
+      <c r="A66" s="13"/>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A67" s="15"/>
+      <c r="A67" s="14"/>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A68" s="16"/>
+      <c r="A68" s="15"/>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A69" s="15"/>
+      <c r="A69" s="14"/>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A70" s="15"/>
+      <c r="A70" s="14"/>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A71" s="17"/>
+      <c r="A71" s="16"/>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A72" s="15"/>
+      <c r="A72" s="14"/>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A73" s="16"/>
+      <c r="A73" s="15"/>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A74" s="15"/>
+      <c r="A74" s="14"/>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A75" s="15"/>
+      <c r="A75" s="14"/>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A76" s="17"/>
+      <c r="A76" s="16"/>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A77" s="17"/>
+      <c r="A77" s="16"/>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A78" s="21"/>
+      <c r="A78" s="20"/>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A79" s="21"/>
+      <c r="A79" s="20"/>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.75">
-      <c r="A80" s="19"/>
+      <c r="A80" s="18"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A81" s="19"/>
+      <c r="A81" s="18"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A82" s="19"/>
+      <c r="A82" s="18"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A83" s="19"/>
+      <c r="A83" s="18"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A84" s="19"/>
+      <c r="A84" s="18"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A85" s="17"/>
+      <c r="A85" s="16"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A86" s="13"/>
+      <c r="A86" s="12"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
       <c r="D86" s="1"/>
@@ -1869,31 +1956,31 @@
       <c r="F87" s="8"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A88" s="15"/>
+      <c r="A88" s="14"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A89" s="16"/>
+      <c r="A89" s="15"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A90" s="15"/>
+      <c r="A90" s="14"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A91" s="15"/>
+      <c r="A91" s="14"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A92" s="17"/>
+      <c r="A92" s="16"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A93" s="18"/>
+      <c r="A93" s="17"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.75">
-      <c r="A94" s="18"/>
+      <c r="A94" s="17"/>
     </row>
     <row r="96" spans="1:6" ht="24.25" x14ac:dyDescent="0.75">
-      <c r="A96" s="14"/>
+      <c r="A96" s="13"/>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A98" s="13"/>
+      <c r="A98" s="12"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
       <c r="D98" s="1"/>
@@ -1902,7 +1989,7 @@
       <c r="G98" s="1"/>
       <c r="H98" s="1"/>
       <c r="I98" s="1"/>
-      <c r="J98" s="22"/>
+      <c r="J98" s="21"/>
       <c r="K98" s="9"/>
       <c r="L98" s="1"/>
       <c r="M98" s="1"/>
@@ -1918,32 +2005,32 @@
       <c r="G99" s="2"/>
       <c r="H99" s="6"/>
       <c r="I99" s="2"/>
-      <c r="J99" s="24"/>
+      <c r="J99" s="23"/>
       <c r="K99" s="11"/>
       <c r="L99" s="2"/>
       <c r="M99" s="5"/>
       <c r="N99" s="11"/>
     </row>
     <row r="101" spans="1:14" ht="24.25" x14ac:dyDescent="0.75">
-      <c r="A101" s="14"/>
+      <c r="A101" s="13"/>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A102" s="15"/>
+      <c r="A102" s="14"/>
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A103" s="16"/>
+      <c r="A103" s="15"/>
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A104" s="16"/>
+      <c r="A104" s="15"/>
     </row>
     <row r="105" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A105" s="16"/>
+      <c r="A105" s="15"/>
     </row>
     <row r="106" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A106" s="16"/>
+      <c r="A106" s="15"/>
     </row>
     <row r="107" spans="1:14" x14ac:dyDescent="0.75">
-      <c r="A107" s="16"/>
+      <c r="A107" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>